<commit_message>
feat: fases 1-3 de importación, geocoding, zonificación, planificación y routing
Incluye backend (imports, overlay de geocoding, zoning, planning, TSP/VRPTW),
frontend, migraciones Alembic, tests e2e y documentación viva.
</commit_message>
<xml_diff>
--- a/docs/requisitos/direcciones-ejemplo-bizkaia.xlsx
+++ b/docs/requisitos/direcciones-ejemplo-bizkaia.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Calle Zabalbide 90, Bajo</t>
+          <t>Calle Zabalbide 92, Bajo</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -614,12 +614,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Calle Iturribide 55, 4º</t>
+          <t>Calle Iturribide 54, 4º</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>48005</t>
+          <t>48006</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Calle Kirikiño 3, Bajo</t>
+          <t>Avenida Kirikiño 2, Bajo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>48004</t>
+          <t>48012</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>48001</t>
+          <t>48009</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Barrio Lezama-Zamudio 8</t>
+          <t>Galbarriatu</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>48170</t>
+          <t>48160</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Barrio Bengoetxe 4</t>
+          <t>Barrio Bengoetxe 5</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2020,12 +2020,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Barrio Mañaria Auzoa 3</t>
+          <t>Aldebaraieta</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>48220</t>
+          <t>48212</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Barrio Elorrio Auzoa 9</t>
+          <t>Berrio</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Calle Foru Kalea 4</t>
+          <t>Besoita</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2131,12 +2131,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Barrio Zaldua 6</t>
+          <t>Sallabente</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>48250</t>
+          <t>48260</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2168,12 +2168,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Barrio Iurreta Auzoa 11</t>
+          <t>Santa Apolonia</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>48260</t>
+          <t>48215</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2205,12 +2205,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Barrio Abadiño Auzoa 7</t>
+          <t>Irazola Auzoa</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>48220</t>
+          <t>48291</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Barrio Muxika Auzoa 5</t>
+          <t>Luparia</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Barrio Arratzu Auzoa 2</t>
+          <t>Zubiate</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>48320</t>
+          <t>48383</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2427,7 +2427,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Barrio Ereño Auzoa 4</t>
+          <t>Gabika</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2464,12 +2464,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Barrio Ibarrangelu Auzoa 1</t>
+          <t>Allika</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>48314</t>
+          <t>48311</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2649,12 +2649,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Barrio Sukarrieta Auzoa 2</t>
+          <t>Abaroa</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>48365</t>
+          <t>48395</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">

</xml_diff>